<commit_message>
Update canteen-e2e.cjs fixes, add apk to gitignore, and sync test reports
</commit_message>
<xml_diff>
--- a/appium-tests/appium-report.xlsx
+++ b/appium-tests/appium-report.xlsx
@@ -34,7 +34,7 @@
     <t>100%</t>
   </si>
   <si>
-    <t>16.69</t>
+    <t>13.48</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -743,7 +743,7 @@
         <v>17</v>
       </c>
       <c r="F8" s="12">
-        <v>1519</v>
+        <v>1389</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>18</v>
@@ -763,7 +763,7 @@
         <v>17</v>
       </c>
       <c r="F9" s="12">
-        <v>1411</v>
+        <v>1475</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>18</v>
@@ -783,7 +783,7 @@
         <v>17</v>
       </c>
       <c r="F10" s="12">
-        <v>1950</v>
+        <v>1726</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>18</v>
@@ -803,7 +803,7 @@
         <v>17</v>
       </c>
       <c r="F11" s="12">
-        <v>1424</v>
+        <v>1319</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>18</v>
@@ -823,7 +823,7 @@
         <v>17</v>
       </c>
       <c r="F12" s="12">
-        <v>1741</v>
+        <v>1606</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>18</v>
@@ -843,7 +843,7 @@
         <v>17</v>
       </c>
       <c r="F13" s="12">
-        <v>1286</v>
+        <v>2007</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>18</v>
@@ -863,7 +863,7 @@
         <v>17</v>
       </c>
       <c r="F14" s="12">
-        <v>1759</v>
+        <v>1399</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>18</v>

</xml_diff>